<commit_message>
Tracker: Status dropdown, phase 2 done
</commit_message>
<xml_diff>
--- a/tracker_template.xlsx
+++ b/tracker_template.xlsx
@@ -808,6 +808,11 @@
       <formula>$AN2="Got it"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="AN2:AN1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"New,Drafted,On hold (trick Q),Needs review,Approved,Sent,Replied,Viewing,Rejected,Got it"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>